<commit_message>
update the excel sheet and align cases (ref_id lowercase, name uppercase)
</commit_message>
<xml_diff>
--- a/tools/excel/bio2/bio2.xlsx
+++ b/tools/excel/bio2/bio2.xlsx
@@ -58,7 +58,7 @@
 6. De bevordering van het beveiligingsbewustzijn.</t>
   </si>
   <si>
-    <t>Basishygiëne, ketenhygiëne</t>
+    <t>Basishygiëne, Ketenhygiëne</t>
   </si>
   <si>
     <t>5.01.02</t>
@@ -378,7 +378,7 @@
     <t>Informatiebeveiligingsincidenten worden afgedaan via het incidentbeheerproces. Ze worden indien relevant gemeld bij toezichthouders volgens de bepalingen uit de betrokken wet- en regelgeving zoals de Cbw, de Archiefwet en de Algemene verordening gegevensbescherming (AVG).</t>
   </si>
   <si>
-    <t>Basishygiëne, overheidsrisico</t>
+    <t>Basishygiëne, Overheidsrisico</t>
   </si>
   <si>
     <t>5.27.01</t>
@@ -898,7 +898,7 @@
     <t>implementation_groups</t>
   </si>
   <si>
-    <t>ketenhygiëne</t>
+    <t>Ketenhygiëne</t>
   </si>
   <si>
     <t>depth</t>
@@ -1932,7 +1932,7 @@
         <v>264</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
fix(lib): align capitalisation in BIO2 implementation groups (#4591)
* Fix BIO2 implementation groups capitalisation

* update the excel sheet and align cases (ref_id lowercase, name uppercase)

* align case convention

* excel sheet

---------

Co-authored-by: Abderrahmane Smimite <smimite@gmail.com>
</commit_message>
<xml_diff>
--- a/tools/excel/bio2/bio2.xlsx
+++ b/tools/excel/bio2/bio2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericlaubacher/Documents/GitHub/ciso-assistant-community/tools/excel/bio2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abder/mydev/intuitem/staging/ciso-assistant-community/tools/excel/bio2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE57CBB3-D588-404B-B0CE-DD3F6A702B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06B9F49-FADA-AE46-8229-C8A965D3B32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20440" activeTab="1" xr2:uid="{51E6D8A9-FAFD-2543-B5A1-6F8F7A044C9B}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20440" activeTab="2" xr2:uid="{51E6D8A9-FAFD-2543-B5A1-6F8F7A044C9B}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="5" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="406">
   <si>
     <t>5.01.01</t>
   </si>
@@ -56,9 +56,6 @@
 4. De gemeenschappelijke betrouwbaarheidseisen en normen die op de organisatie van toepassing zijn.
 5. De frequentie waarmee het informatiebeveiligingsbeleid wordt geëvalueerd.
 6. De bevordering van het beveiligingsbewustzijn.</t>
-  </si>
-  <si>
-    <t>Basishygiëne, ketenhygiëne</t>
   </si>
   <si>
     <t>5.01.02</t>
@@ -378,9 +375,6 @@
     <t>Informatiebeveiligingsincidenten worden afgedaan via het incidentbeheerproces. Ze worden indien relevant gemeld bij toezichthouders volgens de bepalingen uit de betrokken wet- en regelgeving zoals de Cbw, de Archiefwet en de Algemene verordening gegevensbescherming (AVG).</t>
   </si>
   <si>
-    <t>Basishygiëne, overheidsrisico</t>
-  </si>
-  <si>
     <t>5.27.01</t>
   </si>
   <si>
@@ -1432,6 +1426,18 @@
     <t>Baseline Information Security for Government 2 (BIO2)
 24 September 2025, version 1.2 final
 The BIO2 is the successor of the BIO 1.04zv. It is the renewed basic standard for information security within the Dutch government. The BIO2 offers a uniform approach and a common framework of standards for information security within the government, in which risk management is central.</t>
+  </si>
+  <si>
+    <t>basishygiëne</t>
+  </si>
+  <si>
+    <t>overheidsrisico</t>
+  </si>
+  <si>
+    <t>basishygiëne, ketenhygiëne</t>
+  </si>
+  <si>
+    <t>basishygiëne, overheidsrisico</t>
   </si>
 </sst>
 </file>
@@ -1913,106 +1919,106 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B4" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B6" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="68" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="119" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B9" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B10" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="57" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="119" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
   </sheetData>
@@ -2031,74 +2037,74 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="99" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B6" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B7" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B8" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="119" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -2123,27 +2129,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E1" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="F1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="9" customFormat="1" ht="195" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B2" s="9">
         <v>1</v>
@@ -2152,2393 +2158,2393 @@
         <v>0</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>1</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="F3" s="12" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="65" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="F4" s="7" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="F5" s="12" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="52" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="F6" s="7" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="F7" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="F8" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="F9" s="7" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="F10" s="12" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="78" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="F11" s="7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="F12" s="7" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="65" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="F13" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="65" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="F14" s="7" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="F15" s="7" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="F16" s="7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B17">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="F17" s="7" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="F18" s="7" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="F19" s="7" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="F20" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="221" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="F21" s="7" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="F22" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="F23" s="7" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="F24" s="7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B25">
         <v>1</v>
       </c>
       <c r="C25" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>51</v>
-      </c>
       <c r="F25" s="7" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="F26" s="7" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B27">
         <v>1</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F27" s="7" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="52" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B28">
         <v>1</v>
       </c>
       <c r="C28" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="F28" s="7" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="78" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="F29" s="7" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="65" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="F30" s="7" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="F31" s="7" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B32">
         <v>1</v>
       </c>
       <c r="C32" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="F32" s="7" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B33">
         <v>1</v>
       </c>
       <c r="C33" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E33" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D33" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="F33" s="7" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B34">
         <v>1</v>
       </c>
       <c r="C34" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E34" s="3" t="s">
+      <c r="F34" s="7" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="52" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>256</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F34" s="7" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="39" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>258</v>
-      </c>
-      <c r="B35">
-        <v>1</v>
-      </c>
-      <c r="C35" s="1" t="s">
+      <c r="D35" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D35" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>71</v>
-      </c>
       <c r="F35" s="7" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B36">
         <v>1</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="F36" s="7" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="52" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B37">
         <v>1</v>
       </c>
       <c r="C37" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E37" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D37" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>75</v>
-      </c>
       <c r="F37" s="7" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B38">
         <v>1</v>
       </c>
       <c r="C38" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="E38" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D38" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="F38" s="7" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="91" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B39">
         <v>1</v>
       </c>
       <c r="C39" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="D39" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="F39" s="7" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B40">
         <v>1</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="E40" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D40" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>81</v>
-      </c>
       <c r="F40" s="7" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B41">
         <v>1</v>
       </c>
       <c r="C41" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="E41" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>83</v>
-      </c>
       <c r="F41" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B42">
         <v>1</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="E42" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D42" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>85</v>
-      </c>
       <c r="F42" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B43">
         <v>1</v>
       </c>
       <c r="C43" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D43" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>87</v>
-      </c>
       <c r="F43" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B44">
         <v>1</v>
       </c>
       <c r="C44" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="E44" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D44" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>89</v>
-      </c>
       <c r="F44" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="78" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B45">
         <v>1</v>
       </c>
       <c r="C45" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="E45" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D45" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>91</v>
-      </c>
       <c r="F45" s="7" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="68" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B46">
         <v>1</v>
       </c>
       <c r="C46" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="E46" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D46" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="F46" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B47">
         <v>1</v>
       </c>
       <c r="C47" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="E47" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D47" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="F47" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B48">
         <v>1</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F48" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B49">
         <v>1</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F49" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B50">
         <v>1</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F50" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B51">
         <v>1</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F51" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B52">
         <v>1</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F52" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B53">
         <v>1</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B54">
         <v>1</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F54" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B55">
         <v>1</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F55" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="52" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B56">
         <v>1</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F56" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B57">
         <v>1</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>96</v>
+        <v>405</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B58">
         <v>1</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B59">
         <v>1</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F59" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B60">
         <v>1</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F60" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B61">
         <v>1</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F61" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B62">
         <v>1</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B63">
         <v>1</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F63" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B64">
         <v>1</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F64" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B65">
         <v>1</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F65" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B66">
         <v>1</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F66" s="13" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B67">
         <v>1</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="85" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B68">
         <v>1</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F68" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B69">
         <v>1</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F69" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="85" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B70">
         <v>1</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F70" s="7" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B71">
         <v>1</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B72">
         <v>1</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F72" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B73">
         <v>1</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F73" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B74">
         <v>1</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F74" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B75">
         <v>1</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B76">
         <v>1</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F76" s="7" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B77">
         <v>1</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B78">
         <v>1</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F78" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="78" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B79">
         <v>1</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B80">
         <v>1</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F80" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B81">
         <v>1</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F81" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B82">
         <v>1</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F82" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="52" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B83">
         <v>1</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F83" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="85" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B84">
         <v>1</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F84" s="7" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="85" spans="1:6" ht="52" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B85">
         <v>1</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F85" s="7" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="86" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B86">
         <v>1</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F86" s="7" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="87" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B87">
         <v>1</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F87" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="88" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B88">
         <v>1</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F88" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B89">
         <v>1</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F89" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B90">
         <v>1</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F90" s="7" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B91">
         <v>1</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F91" s="7" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B92">
         <v>1</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F92" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B93">
         <v>1</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F93" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="94" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B94">
         <v>1</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F94" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B95">
         <v>1</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F95" s="7" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="96" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B96">
         <v>1</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>96</v>
+        <v>405</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F96" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="97" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B97">
         <v>1</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F97" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="98" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B98">
         <v>1</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F98" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B99">
         <v>1</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E99" s="5" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F99" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="100" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B100">
         <v>1</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F100" s="7" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="101" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B101">
         <v>1</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F101" s="7" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B102">
         <v>1</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F102" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="103" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B103">
         <v>1</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F103" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="104" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B104">
         <v>1</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F104" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="105" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B105">
         <v>1</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F105" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B106">
         <v>1</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F106" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B107">
         <v>1</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F107" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="108" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B108">
         <v>1</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F108" s="7" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B109">
         <v>1</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F109" s="12" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="110" spans="1:6" ht="136" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B110">
         <v>1</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F110" s="7" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B111">
         <v>1</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F111" s="7" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B112">
         <v>1</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F112" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="113" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B113">
         <v>1</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E113" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F113" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="114" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B114">
         <v>1</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F114" s="7" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="115" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B115">
         <v>1</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E115" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="F115" s="7" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="116" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B116">
         <v>1</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F116" s="7" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="117" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B117">
         <v>1</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>2</v>
+        <v>404</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F117" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="118" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B118">
         <v>1</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E118" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="F118" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="119" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B119">
         <v>1</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="F119" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="68" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B120">
         <v>1</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F120" s="7" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B121">
         <v>1</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F121" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -4557,18 +4563,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -4588,46 +4594,46 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C1" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>402</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C3" t="s">
-        <v>255</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>403</v>
       </c>
       <c r="B4" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix wrong IG names in BIO2 and AirCyber
</commit_message>
<xml_diff>
--- a/tools/excel/bio2/bio2.xlsx
+++ b/tools/excel/bio2/bio2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abder/mydev/intuitem/staging/ciso-assistant-community/tools/excel/bio2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericlaubacher/Documents/GitHub/ciso-assistant-community/tools/excel/bio2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06B9F49-FADA-AE46-8229-C8A965D3B32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF447FCE-0ACE-774B-9D41-EE7C0045B561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20440" activeTab="2" xr2:uid="{51E6D8A9-FAFD-2543-B5A1-6F8F7A044C9B}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20440" xr2:uid="{51E6D8A9-FAFD-2543-B5A1-6F8F7A044C9B}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="5" r:id="rId1"/>
@@ -1938,7 +1938,7 @@
         <v>262</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -2298,7 +2298,7 @@
         <v>16</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>18</v>
+        <v>253</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>17</v>
@@ -2318,7 +2318,7 @@
         <v>19</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>18</v>
+        <v>253</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>20</v>
@@ -2807,7 +2807,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="52" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>256</v>
       </c>
@@ -3418,7 +3418,7 @@
         <v>129</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>18</v>
+        <v>253</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>130</v>

</xml_diff>

<commit_message>
fix wrong IG names in BIO2 and AirCyber (#4718)
</commit_message>
<xml_diff>
--- a/tools/excel/bio2/bio2.xlsx
+++ b/tools/excel/bio2/bio2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abder/mydev/intuitem/staging/ciso-assistant-community/tools/excel/bio2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericlaubacher/Documents/GitHub/ciso-assistant-community/tools/excel/bio2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06B9F49-FADA-AE46-8229-C8A965D3B32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF447FCE-0ACE-774B-9D41-EE7C0045B561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20440" activeTab="2" xr2:uid="{51E6D8A9-FAFD-2543-B5A1-6F8F7A044C9B}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20440" xr2:uid="{51E6D8A9-FAFD-2543-B5A1-6F8F7A044C9B}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="5" r:id="rId1"/>
@@ -1938,7 +1938,7 @@
         <v>262</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -2298,7 +2298,7 @@
         <v>16</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>18</v>
+        <v>253</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>17</v>
@@ -2318,7 +2318,7 @@
         <v>19</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>18</v>
+        <v>253</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>20</v>
@@ -2807,7 +2807,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="52" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>256</v>
       </c>
@@ -3418,7 +3418,7 @@
         <v>129</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>18</v>
+        <v>253</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>130</v>

</xml_diff>